<commit_message>
installing gsw for density calculations
</commit_message>
<xml_diff>
--- a/Sal_binned.xlsx
+++ b/Sal_binned.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Steffi Hodnett\MSc_Project\Project_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steph\Project\agg_model_MSc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C034F1A-E1BD-4897-9F13-1A62FBC41DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA936AFE-9084-4240-9DAE-ACA0BCD3F194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4903659" sheetId="1" r:id="rId1"/>
@@ -21,393 +21,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="146">
   <si>
     <t>depth_bin</t>
-  </si>
-  <si>
-    <t>4903659_P1</t>
-  </si>
-  <si>
-    <t>4903659_P10</t>
-  </si>
-  <si>
-    <t>4903659_P11</t>
-  </si>
-  <si>
-    <t>4903659_P12</t>
-  </si>
-  <si>
-    <t>4903659_P14</t>
-  </si>
-  <si>
-    <t>4903659_P15</t>
-  </si>
-  <si>
-    <t>4903659_P16</t>
-  </si>
-  <si>
-    <t>4903659_P17</t>
-  </si>
-  <si>
-    <t>4903659_P18</t>
-  </si>
-  <si>
-    <t>4903659_P19</t>
-  </si>
-  <si>
-    <t>4903659_P2</t>
-  </si>
-  <si>
-    <t>4903659_P20</t>
-  </si>
-  <si>
-    <t>4903659_P21</t>
-  </si>
-  <si>
-    <t>4903659_P22</t>
-  </si>
-  <si>
-    <t>4903659_P23</t>
-  </si>
-  <si>
-    <t>4903659_P24</t>
-  </si>
-  <si>
-    <t>4903659_P25</t>
-  </si>
-  <si>
-    <t>4903659_P26</t>
-  </si>
-  <si>
-    <t>4903659_P27</t>
-  </si>
-  <si>
-    <t>4903659_P28</t>
-  </si>
-  <si>
-    <t>4903659_P29</t>
-  </si>
-  <si>
-    <t>4903659_P3</t>
-  </si>
-  <si>
-    <t>4903659_P30</t>
-  </si>
-  <si>
-    <t>4903659_P31</t>
-  </si>
-  <si>
-    <t>4903659_P32</t>
-  </si>
-  <si>
-    <t>4903659_P33</t>
-  </si>
-  <si>
-    <t>4903659_P34</t>
-  </si>
-  <si>
-    <t>4903659_P35</t>
-  </si>
-  <si>
-    <t>4903659_P36</t>
-  </si>
-  <si>
-    <t>4903659_P37</t>
-  </si>
-  <si>
-    <t>4903659_P38</t>
-  </si>
-  <si>
-    <t>4903659_P39</t>
-  </si>
-  <si>
-    <t>4903659_P4</t>
-  </si>
-  <si>
-    <t>4903659_P40</t>
-  </si>
-  <si>
-    <t>4903659_P41</t>
-  </si>
-  <si>
-    <t>4903659_P42</t>
-  </si>
-  <si>
-    <t>4903659_P43</t>
-  </si>
-  <si>
-    <t>4903659_P44</t>
-  </si>
-  <si>
-    <t>4903659_P5</t>
-  </si>
-  <si>
-    <t>4903659_P6</t>
-  </si>
-  <si>
-    <t>4903659_P7</t>
-  </si>
-  <si>
-    <t>4903659_P8</t>
-  </si>
-  <si>
-    <t>4903659_P9</t>
-  </si>
-  <si>
-    <t>6990636_P1</t>
-  </si>
-  <si>
-    <t>6990636_P10</t>
-  </si>
-  <si>
-    <t>6990636_P11</t>
-  </si>
-  <si>
-    <t>6990636_P12</t>
-  </si>
-  <si>
-    <t>6990636_P13</t>
-  </si>
-  <si>
-    <t>6990636_P14</t>
-  </si>
-  <si>
-    <t>6990636_P15</t>
-  </si>
-  <si>
-    <t>6990636_P16</t>
-  </si>
-  <si>
-    <t>6990636_P17</t>
-  </si>
-  <si>
-    <t>6990636_P18</t>
-  </si>
-  <si>
-    <t>6990636_P19</t>
-  </si>
-  <si>
-    <t>6990636_P2</t>
-  </si>
-  <si>
-    <t>6990636_P20</t>
-  </si>
-  <si>
-    <t>6990636_P21</t>
-  </si>
-  <si>
-    <t>6990636_P22</t>
-  </si>
-  <si>
-    <t>6990636_P23</t>
-  </si>
-  <si>
-    <t>6990636_P24</t>
-  </si>
-  <si>
-    <t>6990636_P25</t>
-  </si>
-  <si>
-    <t>6990636_P26</t>
-  </si>
-  <si>
-    <t>6990636_P27</t>
-  </si>
-  <si>
-    <t>6990636_P28</t>
-  </si>
-  <si>
-    <t>6990636_P29</t>
-  </si>
-  <si>
-    <t>6990636_P3</t>
-  </si>
-  <si>
-    <t>6990636_P30</t>
-  </si>
-  <si>
-    <t>6990636_P31</t>
-  </si>
-  <si>
-    <t>6990636_P32</t>
-  </si>
-  <si>
-    <t>6990636_P33</t>
-  </si>
-  <si>
-    <t>6990636_P34</t>
-  </si>
-  <si>
-    <t>6990636_P35</t>
-  </si>
-  <si>
-    <t>6990636_P36</t>
-  </si>
-  <si>
-    <t>6990636_P37</t>
-  </si>
-  <si>
-    <t>6990636_P38</t>
-  </si>
-  <si>
-    <t>6990636_P39</t>
-  </si>
-  <si>
-    <t>6990636_P4</t>
-  </si>
-  <si>
-    <t>6990636_P40</t>
-  </si>
-  <si>
-    <t>6990636_P41</t>
-  </si>
-  <si>
-    <t>6990636_P42</t>
-  </si>
-  <si>
-    <t>6990636_P43</t>
-  </si>
-  <si>
-    <t>6990636_P44</t>
-  </si>
-  <si>
-    <t>6990636_P45</t>
-  </si>
-  <si>
-    <t>6990636_P46</t>
-  </si>
-  <si>
-    <t>6990636_P47</t>
-  </si>
-  <si>
-    <t>6990636_P48</t>
-  </si>
-  <si>
-    <t>6990636_P49</t>
-  </si>
-  <si>
-    <t>6990636_P5</t>
-  </si>
-  <si>
-    <t>6990636_P50</t>
-  </si>
-  <si>
-    <t>6990636_P51</t>
-  </si>
-  <si>
-    <t>6990636_P52</t>
-  </si>
-  <si>
-    <t>6990636_P53</t>
-  </si>
-  <si>
-    <t>6990636_P54</t>
-  </si>
-  <si>
-    <t>6990636_P55</t>
-  </si>
-  <si>
-    <t>6990636_P56</t>
-  </si>
-  <si>
-    <t>6990636_P57</t>
-  </si>
-  <si>
-    <t>6990636_P58</t>
-  </si>
-  <si>
-    <t>6990636_P59</t>
-  </si>
-  <si>
-    <t>6990636_P6</t>
-  </si>
-  <si>
-    <t>6990636_P60</t>
-  </si>
-  <si>
-    <t>6990636_P61</t>
-  </si>
-  <si>
-    <t>6990636_P62</t>
-  </si>
-  <si>
-    <t>6990636_P63</t>
-  </si>
-  <si>
-    <t>6990636_P64</t>
-  </si>
-  <si>
-    <t>6990636_P65</t>
-  </si>
-  <si>
-    <t>6990636_P66</t>
-  </si>
-  <si>
-    <t>6990636_P67</t>
-  </si>
-  <si>
-    <t>6990636_P68</t>
-  </si>
-  <si>
-    <t>6990636_P69</t>
-  </si>
-  <si>
-    <t>6990636_P7</t>
-  </si>
-  <si>
-    <t>6990636_P70</t>
-  </si>
-  <si>
-    <t>6990636_P71</t>
-  </si>
-  <si>
-    <t>6990636_P73</t>
-  </si>
-  <si>
-    <t>6990636_P74</t>
-  </si>
-  <si>
-    <t>6990636_P75</t>
-  </si>
-  <si>
-    <t>6990636_P76</t>
-  </si>
-  <si>
-    <t>6990636_P77</t>
-  </si>
-  <si>
-    <t>6990636_P78</t>
-  </si>
-  <si>
-    <t>6990636_P79</t>
-  </si>
-  <si>
-    <t>6990636_P8</t>
-  </si>
-  <si>
-    <t>6990636_P80</t>
-  </si>
-  <si>
-    <t>6990636_P81</t>
-  </si>
-  <si>
-    <t>6990636_P82</t>
-  </si>
-  <si>
-    <t>6990636_P83</t>
-  </si>
-  <si>
-    <t>6990636_P84</t>
-  </si>
-  <si>
-    <t>6990636_P85</t>
-  </si>
-  <si>
-    <t>6990636_P86</t>
-  </si>
-  <si>
-    <t>6990636_P9</t>
   </si>
   <si>
     <t>0–10</t>
@@ -588,6 +204,261 @@
   </si>
   <si>
     <t>1950–2000</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>P10</t>
+  </si>
+  <si>
+    <t>P11</t>
+  </si>
+  <si>
+    <t>P12</t>
+  </si>
+  <si>
+    <t>P14</t>
+  </si>
+  <si>
+    <t>P15</t>
+  </si>
+  <si>
+    <t>P16</t>
+  </si>
+  <si>
+    <t>P17</t>
+  </si>
+  <si>
+    <t>P18</t>
+  </si>
+  <si>
+    <t>P19</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>P20</t>
+  </si>
+  <si>
+    <t>P21</t>
+  </si>
+  <si>
+    <t>P22</t>
+  </si>
+  <si>
+    <t>P23</t>
+  </si>
+  <si>
+    <t>P24</t>
+  </si>
+  <si>
+    <t>P25</t>
+  </si>
+  <si>
+    <t>P26</t>
+  </si>
+  <si>
+    <t>P27</t>
+  </si>
+  <si>
+    <t>P28</t>
+  </si>
+  <si>
+    <t>P29</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>P30</t>
+  </si>
+  <si>
+    <t>P31</t>
+  </si>
+  <si>
+    <t>P32</t>
+  </si>
+  <si>
+    <t>P33</t>
+  </si>
+  <si>
+    <t>P34</t>
+  </si>
+  <si>
+    <t>P35</t>
+  </si>
+  <si>
+    <t>P36</t>
+  </si>
+  <si>
+    <t>P37</t>
+  </si>
+  <si>
+    <t>P38</t>
+  </si>
+  <si>
+    <t>P39</t>
+  </si>
+  <si>
+    <t>P4</t>
+  </si>
+  <si>
+    <t>P40</t>
+  </si>
+  <si>
+    <t>P41</t>
+  </si>
+  <si>
+    <t>P42</t>
+  </si>
+  <si>
+    <t>P43</t>
+  </si>
+  <si>
+    <t>P44</t>
+  </si>
+  <si>
+    <t>P5</t>
+  </si>
+  <si>
+    <t>P6</t>
+  </si>
+  <si>
+    <t>P7</t>
+  </si>
+  <si>
+    <t>P8</t>
+  </si>
+  <si>
+    <t>P9</t>
+  </si>
+  <si>
+    <t>P13</t>
+  </si>
+  <si>
+    <t>P45</t>
+  </si>
+  <si>
+    <t>P46</t>
+  </si>
+  <si>
+    <t>P47</t>
+  </si>
+  <si>
+    <t>P48</t>
+  </si>
+  <si>
+    <t>P49</t>
+  </si>
+  <si>
+    <t>P50</t>
+  </si>
+  <si>
+    <t>P51</t>
+  </si>
+  <si>
+    <t>P52</t>
+  </si>
+  <si>
+    <t>P53</t>
+  </si>
+  <si>
+    <t>P54</t>
+  </si>
+  <si>
+    <t>P55</t>
+  </si>
+  <si>
+    <t>P56</t>
+  </si>
+  <si>
+    <t>P57</t>
+  </si>
+  <si>
+    <t>P58</t>
+  </si>
+  <si>
+    <t>P59</t>
+  </si>
+  <si>
+    <t>P60</t>
+  </si>
+  <si>
+    <t>P61</t>
+  </si>
+  <si>
+    <t>P62</t>
+  </si>
+  <si>
+    <t>P63</t>
+  </si>
+  <si>
+    <t>P64</t>
+  </si>
+  <si>
+    <t>P65</t>
+  </si>
+  <si>
+    <t>P66</t>
+  </si>
+  <si>
+    <t>P67</t>
+  </si>
+  <si>
+    <t>P68</t>
+  </si>
+  <si>
+    <t>P69</t>
+  </si>
+  <si>
+    <t>P70</t>
+  </si>
+  <si>
+    <t>P71</t>
+  </si>
+  <si>
+    <t>P73</t>
+  </si>
+  <si>
+    <t>P74</t>
+  </si>
+  <si>
+    <t>P75</t>
+  </si>
+  <si>
+    <t>P76</t>
+  </si>
+  <si>
+    <t>P77</t>
+  </si>
+  <si>
+    <t>P78</t>
+  </si>
+  <si>
+    <t>P79</t>
+  </si>
+  <si>
+    <t>P80</t>
+  </si>
+  <si>
+    <t>P81</t>
+  </si>
+  <si>
+    <t>P82</t>
+  </si>
+  <si>
+    <t>P83</t>
+  </si>
+  <si>
+    <t>P84</t>
+  </si>
+  <si>
+    <t>P85</t>
+  </si>
+  <si>
+    <t>P86</t>
   </si>
 </sst>
 </file>
@@ -966,133 +837,133 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>63</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>66</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>67</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>69</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>71</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>73</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>16</v>
+        <v>76</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>19</v>
+        <v>79</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>22</v>
+        <v>82</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>23</v>
+        <v>83</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>27</v>
+        <v>87</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>28</v>
+        <v>88</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>31</v>
+        <v>91</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>32</v>
+        <v>92</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>33</v>
+        <v>93</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>34</v>
+        <v>94</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>36</v>
+        <v>96</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>38</v>
+        <v>98</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>41</v>
+        <v>101</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>42</v>
+        <v>102</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>43</v>
+        <v>103</v>
       </c>
       <c r="AS1" s="1"/>
       <c r="AT1" s="1"/>
@@ -1182,7 +1053,7 @@
     </row>
     <row r="2" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>129</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <v>35.171504811320752</v>
@@ -1316,7 +1187,7 @@
     </row>
     <row r="3" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <v>35.171575411764707</v>
@@ -1447,7 +1318,7 @@
     </row>
     <row r="4" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>131</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>35.171367687500002</v>
@@ -1578,7 +1449,7 @@
     </row>
     <row r="5" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>132</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>35.171019800000003</v>
@@ -1709,7 +1580,7 @@
     </row>
     <row r="6" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>133</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>35.174715999999997</v>
@@ -1840,7 +1711,7 @@
     </row>
     <row r="7" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>134</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>35.181823933333327</v>
@@ -1971,7 +1842,7 @@
     </row>
     <row r="8" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>135</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>35.182827533333338</v>
@@ -2102,7 +1973,7 @@
     </row>
     <row r="9" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>136</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <v>35.190432000000001</v>
@@ -2233,7 +2104,7 @@
     </row>
     <row r="10" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>137</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <v>35.196327750000002</v>
@@ -2364,7 +2235,7 @@
     </row>
     <row r="11" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>138</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <v>35.195276999999997</v>
@@ -2495,7 +2366,7 @@
     </row>
     <row r="12" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>139</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <v>35.210381903225809</v>
@@ -2626,7 +2497,7 @@
     </row>
     <row r="13" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>35.2180859375</v>
@@ -2757,7 +2628,7 @@
     </row>
     <row r="14" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>141</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>35.217208451612898</v>
@@ -2888,7 +2759,7 @@
     </row>
     <row r="15" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>142</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>35.199731096774187</v>
@@ -3019,7 +2890,7 @@
     </row>
     <row r="16" spans="1:129" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>143</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>35.196589633333332</v>
@@ -3150,7 +3021,7 @@
     </row>
     <row r="17" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>144</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>35.187525580645158</v>
@@ -3281,7 +3152,7 @@
     </row>
     <row r="18" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>145</v>
+        <v>17</v>
       </c>
       <c r="B18">
         <v>35.190119470588243</v>
@@ -3412,7 +3283,7 @@
     </row>
     <row r="19" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>146</v>
+        <v>18</v>
       </c>
       <c r="B19">
         <v>35.204791515151513</v>
@@ -3543,7 +3414,7 @@
     </row>
     <row r="20" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>147</v>
+        <v>19</v>
       </c>
       <c r="B20">
         <v>35.18816546875</v>
@@ -3674,7 +3545,7 @@
     </row>
     <row r="21" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>148</v>
+        <v>20</v>
       </c>
       <c r="B21">
         <v>35.188809249999998</v>
@@ -3805,7 +3676,7 @@
     </row>
     <row r="22" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>149</v>
+        <v>21</v>
       </c>
       <c r="B22">
         <v>35.186780260869561</v>
@@ -3936,7 +3807,7 @@
     </row>
     <row r="23" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>150</v>
+        <v>22</v>
       </c>
       <c r="B23">
         <v>35.172840399999998</v>
@@ -4067,7 +3938,7 @@
     </row>
     <row r="24" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>151</v>
+        <v>23</v>
       </c>
       <c r="B24">
         <v>35.168148041666669</v>
@@ -4198,7 +4069,7 @@
     </row>
     <row r="25" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>152</v>
+        <v>24</v>
       </c>
       <c r="B25">
         <v>35.183248124999999</v>
@@ -4329,7 +4200,7 @@
     </row>
     <row r="26" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>153</v>
+        <v>25</v>
       </c>
       <c r="B26">
         <v>35.193756695652183</v>
@@ -4460,7 +4331,7 @@
     </row>
     <row r="27" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>154</v>
+        <v>26</v>
       </c>
       <c r="B27">
         <v>35.183690636363643</v>
@@ -4591,7 +4462,7 @@
     </row>
     <row r="28" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>155</v>
+        <v>27</v>
       </c>
       <c r="B28">
         <v>35.18547977272727</v>
@@ -4722,7 +4593,7 @@
     </row>
     <row r="29" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>156</v>
+        <v>28</v>
       </c>
       <c r="B29">
         <v>35.183585727272728</v>
@@ -4853,7 +4724,7 @@
     </row>
     <row r="30" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>157</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>35.160437999999999</v>
@@ -4984,7 +4855,7 @@
     </row>
     <row r="31" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>158</v>
+        <v>30</v>
       </c>
       <c r="B31">
         <v>35.142862583333333</v>
@@ -5112,7 +4983,7 @@
     </row>
     <row r="32" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>159</v>
+        <v>31</v>
       </c>
       <c r="B32">
         <v>35.119614385964908</v>
@@ -5243,7 +5114,7 @@
     </row>
     <row r="33" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>160</v>
+        <v>32</v>
       </c>
       <c r="B33">
         <v>35.095805622950813</v>
@@ -5374,7 +5245,7 @@
     </row>
     <row r="34" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>161</v>
+        <v>33</v>
       </c>
       <c r="B34">
         <v>35.092977098360649</v>
@@ -5505,7 +5376,7 @@
     </row>
     <row r="35" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>162</v>
+        <v>34</v>
       </c>
       <c r="B35">
         <v>35.060772290909092</v>
@@ -5636,7 +5507,7 @@
     </row>
     <row r="36" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>163</v>
+        <v>35</v>
       </c>
       <c r="B36">
         <v>35.031231523809517</v>
@@ -5767,7 +5638,7 @@
     </row>
     <row r="37" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>164</v>
+        <v>36</v>
       </c>
       <c r="B37">
         <v>35.002818830508467</v>
@@ -5898,7 +5769,7 @@
     </row>
     <row r="38" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>165</v>
+        <v>37</v>
       </c>
       <c r="B38">
         <v>34.982568629032258</v>
@@ -6029,7 +5900,7 @@
     </row>
     <row r="39" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>166</v>
+        <v>38</v>
       </c>
       <c r="B39">
         <v>34.966343344827592</v>
@@ -6160,7 +6031,7 @@
     </row>
     <row r="40" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>167</v>
+        <v>39</v>
       </c>
       <c r="B40">
         <v>34.955527406779659</v>
@@ -6291,7 +6162,7 @@
     </row>
     <row r="41" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>168</v>
+        <v>40</v>
       </c>
       <c r="B41">
         <v>34.9460083559322</v>
@@ -6422,7 +6293,7 @@
     </row>
     <row r="42" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>169</v>
+        <v>41</v>
       </c>
       <c r="B42">
         <v>34.940316500000002</v>
@@ -6535,7 +6406,7 @@
     </row>
     <row r="43" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>170</v>
+        <v>42</v>
       </c>
       <c r="L43">
         <v>34.930107999999997</v>
@@ -6621,7 +6492,7 @@
     </row>
     <row r="44" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>171</v>
+        <v>43</v>
       </c>
       <c r="L44">
         <v>34.922138750000002</v>
@@ -6707,7 +6578,7 @@
     </row>
     <row r="45" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>172</v>
+        <v>44</v>
       </c>
       <c r="L45">
         <v>34.918784000000002</v>
@@ -6793,7 +6664,7 @@
     </row>
     <row r="46" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>173</v>
+        <v>45</v>
       </c>
       <c r="L46">
         <v>34.914202000000003</v>
@@ -6879,7 +6750,7 @@
     </row>
     <row r="47" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="L47">
         <v>34.909152749999997</v>
@@ -6965,7 +6836,7 @@
     </row>
     <row r="48" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>175</v>
+        <v>47</v>
       </c>
       <c r="L48">
         <v>34.906095333333333</v>
@@ -7051,7 +6922,7 @@
     </row>
     <row r="49" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>176</v>
+        <v>48</v>
       </c>
       <c r="L49">
         <v>34.904021749999998</v>
@@ -7137,7 +7008,7 @@
     </row>
     <row r="50" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>177</v>
+        <v>49</v>
       </c>
       <c r="L50">
         <v>34.901056250000003</v>
@@ -7223,7 +7094,7 @@
     </row>
     <row r="51" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>178</v>
+        <v>50</v>
       </c>
       <c r="L51">
         <v>34.899258666666668</v>
@@ -7309,7 +7180,7 @@
     </row>
     <row r="52" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>179</v>
+        <v>51</v>
       </c>
       <c r="L52">
         <v>34.901033750000003</v>
@@ -7395,7 +7266,7 @@
     </row>
     <row r="53" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>180</v>
+        <v>52</v>
       </c>
       <c r="L53">
         <v>34.907732000000003</v>
@@ -7481,7 +7352,7 @@
     </row>
     <row r="54" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>181</v>
+        <v>53</v>
       </c>
       <c r="L54">
         <v>34.923852749999988</v>
@@ -7567,7 +7438,7 @@
     </row>
     <row r="55" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>182</v>
+        <v>54</v>
       </c>
       <c r="L55">
         <v>34.939640666666669</v>
@@ -7653,7 +7524,7 @@
     </row>
     <row r="56" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>183</v>
+        <v>55</v>
       </c>
       <c r="L56">
         <v>34.950885999999997</v>
@@ -7739,7 +7610,7 @@
     </row>
     <row r="57" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>184</v>
+        <v>56</v>
       </c>
       <c r="L57">
         <v>34.954935749999997</v>
@@ -7825,7 +7696,7 @@
     </row>
     <row r="58" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>185</v>
+        <v>57</v>
       </c>
       <c r="L58">
         <v>34.949925333333333</v>
@@ -7908,7 +7779,7 @@
     </row>
     <row r="59" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>186</v>
+        <v>58</v>
       </c>
       <c r="L59">
         <v>34.955375250000003</v>
@@ -7988,7 +7859,7 @@
     </row>
     <row r="60" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>187</v>
+        <v>59</v>
       </c>
       <c r="L60">
         <v>34.958383499999997</v>
@@ -8065,7 +7936,7 @@
     </row>
     <row r="61" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>188</v>
+        <v>60</v>
       </c>
       <c r="L61">
         <v>34.964875999999997</v>
@@ -8153,264 +8024,264 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>104</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>53</v>
+        <v>69</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>55</v>
+        <v>71</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>59</v>
+        <v>75</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="AN1" s="1" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>84</v>
+        <v>106</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>85</v>
+        <v>107</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>86</v>
+        <v>108</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>93</v>
+        <v>114</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
       <c r="BB1" s="1" t="s">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="BC1" s="1" t="s">
-        <v>97</v>
+        <v>118</v>
       </c>
       <c r="BD1" s="1" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="BF1" s="1" t="s">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="BG1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="BH1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="BI1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="BJ1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="BK1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="BL1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="BM1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="BN1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="BO1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="BP1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="BH1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="BR1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="BS1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="BT1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="BU1" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="BV1" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="BW1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="BX1" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="BY1" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="BZ1" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="BI1" s="1" t="s">
+      <c r="CA1" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="CB1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="CC1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="CD1" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="CE1" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="CF1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="CG1" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="CH1" s="1" t="s">
         <v>103</v>
-      </c>
-      <c r="BJ1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="BK1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="BL1" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="BM1" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="BN1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="BO1" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="BP1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="BQ1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="BR1" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="BS1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="BT1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="BU1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="BV1" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="BW1" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="BX1" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="BY1" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="BZ1" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="CA1" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="CB1" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="CC1" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="CD1" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="CE1" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="CF1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="CG1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="CH1" s="1" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>129</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <v>35.170302086956532</v>
@@ -8670,7 +8541,7 @@
     </row>
     <row r="3" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>130</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <v>35.170403714285712</v>
@@ -8930,7 +8801,7 @@
     </row>
     <row r="4" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>131</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>35.170980999999998</v>
@@ -9190,7 +9061,7 @@
     </row>
     <row r="5" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>132</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>35.170974999999999</v>
@@ -9450,7 +9321,7 @@
     </row>
     <row r="6" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>133</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>35.175189812500001</v>
@@ -9710,7 +9581,7 @@
     </row>
     <row r="7" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>134</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>35.186673533333327</v>
@@ -9970,7 +9841,7 @@
     </row>
     <row r="8" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>135</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>35.188997624999999</v>
@@ -10230,7 +10101,7 @@
     </row>
     <row r="9" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>136</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <v>35.188956666666662</v>
@@ -10490,7 +10361,7 @@
     </row>
     <row r="10" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>137</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <v>35.189475199999997</v>
@@ -10750,7 +10621,7 @@
     </row>
     <row r="11" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>138</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <v>35.187377733333328</v>
@@ -11010,7 +10881,7 @@
     </row>
     <row r="12" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>139</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <v>35.180587366666671</v>
@@ -11270,7 +11141,7 @@
     </row>
     <row r="13" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>35.190155322580651</v>
@@ -11530,7 +11401,7 @@
     </row>
     <row r="14" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>141</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>35.189371866666669</v>
@@ -11790,7 +11661,7 @@
     </row>
     <row r="15" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>142</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>35.184564656249997</v>
@@ -12050,7 +11921,7 @@
     </row>
     <row r="16" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>143</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>35.178009000000003</v>
@@ -12310,7 +12181,7 @@
     </row>
     <row r="17" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>144</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>35.178899375</v>
@@ -12570,7 +12441,7 @@
     </row>
     <row r="18" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>145</v>
+        <v>17</v>
       </c>
       <c r="B18">
         <v>35.184330129032261</v>
@@ -12830,7 +12701,7 @@
     </row>
     <row r="19" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>146</v>
+        <v>18</v>
       </c>
       <c r="B19">
         <v>35.190378900000013</v>
@@ -13090,7 +12961,7 @@
     </row>
     <row r="20" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>147</v>
+        <v>19</v>
       </c>
       <c r="B20">
         <v>35.180535499999998</v>
@@ -13350,7 +13221,7 @@
     </row>
     <row r="21" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>148</v>
+        <v>20</v>
       </c>
       <c r="B21">
         <v>35.178106</v>
@@ -13610,7 +13481,7 @@
     </row>
     <row r="22" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>149</v>
+        <v>21</v>
       </c>
       <c r="B22">
         <v>35.176580480000013</v>
@@ -13870,7 +13741,7 @@
     </row>
     <row r="23" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>150</v>
+        <v>22</v>
       </c>
       <c r="B23">
         <v>35.181344500000002</v>
@@ -14130,7 +14001,7 @@
     </row>
     <row r="24" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>151</v>
+        <v>23</v>
       </c>
       <c r="B24">
         <v>35.181244200000002</v>
@@ -14390,7 +14261,7 @@
     </row>
     <row r="25" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>152</v>
+        <v>24</v>
       </c>
       <c r="B25">
         <v>35.169927541666667</v>
@@ -14650,7 +14521,7 @@
     </row>
     <row r="26" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>153</v>
+        <v>25</v>
       </c>
       <c r="B26">
         <v>35.17283316666667</v>
@@ -14910,7 +14781,7 @@
     </row>
     <row r="27" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>154</v>
+        <v>26</v>
       </c>
       <c r="B27">
         <v>35.172872434782597</v>
@@ -15170,7 +15041,7 @@
     </row>
     <row r="28" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>155</v>
+        <v>27</v>
       </c>
       <c r="B28">
         <v>35.185943954545458</v>
@@ -15430,7 +15301,7 @@
     </row>
     <row r="29" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>156</v>
+        <v>28</v>
       </c>
       <c r="B29">
         <v>35.195603318181817</v>
@@ -15690,7 +15561,7 @@
     </row>
     <row r="30" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>157</v>
+        <v>29</v>
       </c>
       <c r="B30">
         <v>35.181256043478257</v>
@@ -15950,7 +15821,7 @@
     </row>
     <row r="31" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>158</v>
+        <v>30</v>
       </c>
       <c r="B31">
         <v>35.165159000000003</v>
@@ -16210,7 +16081,7 @@
     </row>
     <row r="32" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>159</v>
+        <v>31</v>
       </c>
       <c r="B32">
         <v>35.132005966666661</v>
@@ -16470,7 +16341,7 @@
     </row>
     <row r="33" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>160</v>
+        <v>32</v>
       </c>
       <c r="B33">
         <v>35.112204927272728</v>
@@ -16730,7 +16601,7 @@
     </row>
     <row r="34" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>161</v>
+        <v>33</v>
       </c>
       <c r="B34">
         <v>35.09361468253968</v>
@@ -16990,7 +16861,7 @@
     </row>
     <row r="35" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>162</v>
+        <v>34</v>
       </c>
       <c r="B35">
         <v>35.063586491525427</v>
@@ -17250,7 +17121,7 @@
     </row>
     <row r="36" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>163</v>
+        <v>35</v>
       </c>
       <c r="B36">
         <v>35.033348160714283</v>
@@ -17510,7 +17381,7 @@
     </row>
     <row r="37" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>164</v>
+        <v>36</v>
       </c>
       <c r="B37">
         <v>35.007212112903233</v>
@@ -17770,7 +17641,7 @@
     </row>
     <row r="38" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>165</v>
+        <v>37</v>
       </c>
       <c r="B38">
         <v>34.9888105</v>
@@ -18030,7 +17901,7 @@
     </row>
     <row r="39" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>166</v>
+        <v>38</v>
       </c>
       <c r="B39">
         <v>34.971527098360653</v>
@@ -18290,7 +18161,7 @@
     </row>
     <row r="40" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>167</v>
+        <v>39</v>
       </c>
       <c r="B40">
         <v>34.960223322033897</v>
@@ -18550,7 +18421,7 @@
     </row>
     <row r="41" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>168</v>
+        <v>40</v>
       </c>
       <c r="B41">
         <v>34.949995228070179</v>
@@ -18810,7 +18681,7 @@
     </row>
     <row r="42" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>169</v>
+        <v>41</v>
       </c>
       <c r="B42">
         <v>34.944727999999998</v>
@@ -19070,7 +18941,7 @@
     </row>
     <row r="43" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>170</v>
+        <v>42</v>
       </c>
       <c r="C43">
         <v>34.935540000000003</v>
@@ -19327,7 +19198,7 @@
     </row>
     <row r="44" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>171</v>
+        <v>43</v>
       </c>
       <c r="C44">
         <v>34.927999999999997</v>
@@ -19584,7 +19455,7 @@
     </row>
     <row r="45" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>172</v>
+        <v>44</v>
       </c>
       <c r="C45">
         <v>34.922555000000003</v>
@@ -19841,7 +19712,7 @@
     </row>
     <row r="46" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>173</v>
+        <v>45</v>
       </c>
       <c r="C46">
         <v>34.917915333333333</v>
@@ -20098,7 +19969,7 @@
     </row>
     <row r="47" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>174</v>
+        <v>46</v>
       </c>
       <c r="C47">
         <v>34.913211250000003</v>
@@ -20355,7 +20226,7 @@
     </row>
     <row r="48" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>175</v>
+        <v>47</v>
       </c>
       <c r="C48">
         <v>34.9086985</v>
@@ -20612,7 +20483,7 @@
     </row>
     <row r="49" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>176</v>
+        <v>48</v>
       </c>
       <c r="C49">
         <v>34.905116666666657</v>
@@ -20869,7 +20740,7 @@
     </row>
     <row r="50" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>177</v>
+        <v>49</v>
       </c>
       <c r="C50">
         <v>34.902237249999999</v>
@@ -21120,7 +20991,7 @@
     </row>
     <row r="51" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>178</v>
+        <v>50</v>
       </c>
       <c r="C51">
         <v>34.899238250000003</v>
@@ -21368,7 +21239,7 @@
     </row>
     <row r="52" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>179</v>
+        <v>51</v>
       </c>
       <c r="C52">
         <v>34.897931249999999</v>
@@ -21616,7 +21487,7 @@
     </row>
     <row r="53" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>180</v>
+        <v>52</v>
       </c>
       <c r="C53">
         <v>34.89706833333333</v>
@@ -21864,7 +21735,7 @@
     </row>
     <row r="54" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>181</v>
+        <v>53</v>
       </c>
       <c r="C54">
         <v>34.897159000000002</v>
@@ -22112,7 +21983,7 @@
     </row>
     <row r="55" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>182</v>
+        <v>54</v>
       </c>
       <c r="C55">
         <v>34.899430500000001</v>
@@ -22360,7 +22231,7 @@
     </row>
     <row r="56" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>183</v>
+        <v>55</v>
       </c>
       <c r="C56">
         <v>34.902933666666662</v>
@@ -22602,7 +22473,7 @@
     </row>
     <row r="57" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>184</v>
+        <v>56</v>
       </c>
       <c r="C57">
         <v>34.907462000000002</v>
@@ -22844,7 +22715,7 @@
     </row>
     <row r="58" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>185</v>
+        <v>57</v>
       </c>
       <c r="C58">
         <v>34.912225999999997</v>
@@ -23077,7 +22948,7 @@
     </row>
     <row r="59" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>186</v>
+        <v>58</v>
       </c>
       <c r="C59">
         <v>34.917444000000003</v>
@@ -23304,7 +23175,7 @@
     </row>
     <row r="60" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>187</v>
+        <v>59</v>
       </c>
       <c r="C60">
         <v>34.922115666666663</v>
@@ -23516,7 +23387,7 @@
     </row>
     <row r="61" spans="1:86" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>188</v>
+        <v>60</v>
       </c>
       <c r="C61">
         <v>34.926063399999997</v>

</xml_diff>